<commit_message>
Rerun lm eval on zero and few shot aggregates
</commit_message>
<xml_diff>
--- a/results/closed_aggregate_few_shot_final/ilsp__Llama-Krikri-8B-Instruct-v1.5/closed_few_shot_final.xlsx
+++ b/results/closed_aggregate_few_shot_final/ilsp__Llama-Krikri-8B-Instruct-v1.5/closed_few_shot_final.xlsx
@@ -507,10 +507,10 @@
         <v>49</v>
       </c>
       <c r="E3" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.6938775510204082</v>
       </c>
       <c r="F3" t="n">
-        <v>0.06520506636966263</v>
+        <v>0.06652247352247599</v>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
@@ -538,10 +538,10 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>0.6046511627906976</v>
+        <v>0.5930232558139535</v>
       </c>
       <c r="H4" t="n">
-        <v>0.05303141512089016</v>
+        <v>0.05328576389483537</v>
       </c>
       <c r="I4" t="inlineStr"/>
     </row>
@@ -565,10 +565,10 @@
         <v>35</v>
       </c>
       <c r="E5" t="n">
-        <v>0.6</v>
+        <v>0.6285714285714286</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0840168050416806</v>
+        <v>0.08286583553358692</v>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
@@ -594,10 +594,10 @@
         <v>20</v>
       </c>
       <c r="E6" t="n">
-        <v>0.8</v>
+        <v>0.75</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0917662935482247</v>
+        <v>0.09933992677987828</v>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
@@ -681,10 +681,10 @@
         <v>35</v>
       </c>
       <c r="E9" t="n">
-        <v>0.7714285714285715</v>
+        <v>0.7428571428571429</v>
       </c>
       <c r="F9" t="n">
-        <v>0.07201440432144052</v>
+        <v>0.07495496847387484</v>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
@@ -707,13 +707,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E10" t="n">
-        <v>0.4545454545454545</v>
+        <v>0.515625</v>
       </c>
       <c r="F10" t="n">
-        <v>0.06176056549879611</v>
+        <v>0.06296331249416676</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
@@ -736,13 +736,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="E11" t="n">
-        <v>0.4864864864864865</v>
+        <v>0.4761904761904762</v>
       </c>
       <c r="F11" t="n">
-        <v>0.08330289193201319</v>
+        <v>0.07799829681942305</v>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
@@ -765,23 +765,23 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="E12" t="n">
-        <v>0.6657534246575343</v>
+        <v>0.6684782608695652</v>
       </c>
       <c r="F12" t="n">
-        <v>0.02354776731897684</v>
+        <v>0.02369088937515106</v>
       </c>
       <c r="G12" t="n">
-        <v>0.6046511627906976</v>
+        <v>0.5930232558139535</v>
       </c>
       <c r="H12" t="n">
-        <v>0.05303141512089017</v>
+        <v>0.05328576389483537</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>{'exact_match,none': 86, 'exact_match,strict-match': 365}</t>
+          <t>{'exact_match,none': 86, 'exact_match,strict-match': 368}</t>
         </is>
       </c>
     </row>

</xml_diff>